<commit_message>
Added new testcase TS007 & TS008 for Ec2 instance run
</commit_message>
<xml_diff>
--- a/Testdata/Testdata_Addemp.xlsx
+++ b/Testdata/Testdata_Addemp.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{945C4755-0306-4AC1-8A49-87F2F015EF97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E880C3E2-885F-4884-96E5-67F689F4EDE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="192">
   <si>
     <t>TestcaseID</t>
   </si>
@@ -561,15 +561,9 @@
     <t>Transport expense</t>
   </si>
   <si>
-    <t>5000</t>
-  </si>
-  <si>
     <t>Fuel Allowance</t>
   </si>
   <si>
-    <t>500</t>
-  </si>
-  <si>
     <t>Fuel expense</t>
   </si>
   <si>
@@ -577,6 +571,30 @@
   </si>
   <si>
     <t>PIM</t>
+  </si>
+  <si>
+    <t>Accommodation</t>
+  </si>
+  <si>
+    <t>Indian Rupee</t>
+  </si>
+  <si>
+    <t>25-10-2015</t>
+  </si>
+  <si>
+    <t>7500</t>
+  </si>
+  <si>
+    <t>Stay Expense</t>
+  </si>
+  <si>
+    <t>6000</t>
+  </si>
+  <si>
+    <t>400</t>
+  </si>
+  <si>
+    <t>30-11-2014</t>
   </si>
 </sst>
 </file>
@@ -1920,7 +1938,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F0C2D35-2E21-4A8E-AA93-6AD21B3254A2}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="8" width="19.77734375" customWidth="1"/>
@@ -1965,11 +1983,11 @@
       <c r="D2" t="s">
         <v>178</v>
       </c>
-      <c r="E2" t="s">
-        <v>67</v>
+      <c r="E2" s="3" t="s">
+        <v>191</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="G2" t="s">
         <v>179</v>
@@ -1977,16 +1995,39 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D3" t="s">
+        <v>180</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="G3" t="s">
         <v>181</v>
       </c>
-      <c r="E3" t="s">
-        <v>67</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>182</v>
-      </c>
-      <c r="G3" t="s">
-        <v>183</v>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="F4" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="G4" t="s">
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -2004,12 +2045,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>